<commit_message>
Adding the core DuckDB parser
</commit_message>
<xml_diff>
--- a/docs/Objectformat.xlsx
+++ b/docs/Objectformat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\translate\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B26AD4-E3AA-4DCB-851F-3C1C97303AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2048ED23-BA75-4D36-9581-9E03111135DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{15AA336A-D685-4105-A88D-4934FBDDFB83}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="589">
   <si>
     <t>AGGREGATE</t>
   </si>
@@ -1796,6 +1796,15 @@
   </si>
   <si>
     <t>ACCOUNT</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>OLD_PASSWORD</t>
+  </si>
+  <si>
+    <t>SESSION</t>
   </si>
 </sst>
 </file>
@@ -2890,10 +2899,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DC1B666D-F140-4714-8059-03985377C409}" name="Table3" displayName="Table3" ref="A1:B270" totalsRowShown="0">
-  <autoFilter ref="A1:B270" xr:uid="{DC1B666D-F140-4714-8059-03985377C409}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B270">
-    <sortCondition ref="A270"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DC1B666D-F140-4714-8059-03985377C409}" name="Table3" displayName="Table3" ref="A1:B275" totalsRowShown="0">
+  <autoFilter ref="A1:B275" xr:uid="{DC1B666D-F140-4714-8059-03985377C409}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B275">
+    <sortCondition ref="A262:A275"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{071EBA71-6222-4CD8-9B5B-3C606DFEC073}" name="ACCOUNT"/>
@@ -34421,7 +34430,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE606DBE-090B-4F3B-A1C1-67D1A3393634}">
-  <dimension ref="A1:B270"/>
+  <dimension ref="A1:B275"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="35.75" bestFit="1" customWidth="1"/>
@@ -34537,2322 +34546,2367 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
+        <v>AUTHORIZATION : 'AUTHORIZATION' ;</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
         <v>336</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B14" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BEFORE : 'BEFORE' ;</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
         <v>337</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BETWEEN : 'BETWEEN' ;</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
         <v>338</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BIGINT : 'BIGINT' ;</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
         <v>339</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BINARY : 'BINARY' ;</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
         <v>340</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B18" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BLOB : 'BLOB' ;</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
         <v>341</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B19" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BOTH : 'BOTH' ;</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
         <v>342</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B20" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>BY : 'BY' ;</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
         <v>343</v>
       </c>
-      <c r="B20" t="str">
+      <c r="B21" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CALL : 'CALL' ;</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
         <v>344</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B22" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CASCADE : 'CASCADE' ;</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
         <v>345</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B23" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CASE : 'CASE' ;</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
         <v>346</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B24" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CHANGE : 'CHANGE' ;</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
         <v>347</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B25" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CHAR : 'CHAR' ;</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
         <v>348</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B26" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CHARACTER : 'CHARACTER' ;</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
-      <c r="A26" t="s">
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
         <v>349</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B27" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CHECK : 'CHECK' ;</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
-      <c r="A27" t="s">
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
         <v>573</v>
       </c>
-      <c r="B27" s="3" t="str">
+      <c r="B28" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CIPHER : 'CIPHER' ;</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
-      <c r="A28" t="s">
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
         <v>350</v>
       </c>
-      <c r="B28" t="str">
+      <c r="B29" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>COLLATE : 'COLLATE' ;</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
-      <c r="A29" t="s">
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
         <v>351</v>
       </c>
-      <c r="B29" t="str">
+      <c r="B30" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>COLUMN : 'COLUMN' ;</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
-      <c r="A30" t="s">
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
         <v>352</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B31" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CONDITION : 'CONDITION' ;</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
-      <c r="A31" t="s">
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
         <v>294</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B32" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CONSTRAINT : 'CONSTRAINT' ;</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
         <v>353</v>
       </c>
-      <c r="B32" t="str">
+      <c r="B33" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CONTINUE : 'CONTINUE' ;</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
-      <c r="A33" t="s">
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
         <v>354</v>
       </c>
-      <c r="B33" t="str">
+      <c r="B34" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CONVERT : 'CONVERT' ;</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
         <v>355</v>
       </c>
-      <c r="B34" t="str">
+      <c r="B35" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CREATE : 'CREATE' ;</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
-      <c r="A35" t="s">
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
         <v>356</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B36" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CROSS : 'CROSS' ;</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
-      <c r="A36" t="s">
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
         <v>357</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B37" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURRENT_DATE : 'CURRENT_DATE' ;</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
-      <c r="A37" t="s">
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
         <v>358</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B38" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURRENT_ROLE : 'CURRENT_ROLE' ;</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
-      <c r="A38" t="s">
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
         <v>359</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B39" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURRENT_TIME : 'CURRENT_TIME' ;</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
-      <c r="A39" t="s">
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
         <v>360</v>
       </c>
-      <c r="B39" t="str">
+      <c r="B40" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURRENT_TIMESTAMP : 'CURRENT_TIMESTAMP' ;</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
-      <c r="A40" t="s">
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
         <v>361</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B41" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURRENT_USER : 'CURRENT_USER' ;</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
         <v>362</v>
       </c>
-      <c r="B41" t="str">
+      <c r="B42" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>CURSOR : 'CURSOR' ;</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
-      <c r="A42" t="s">
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
         <v>13</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B43" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DATABASE : 'DATABASE' ;</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
-      <c r="A43" t="s">
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
         <v>363</v>
       </c>
-      <c r="B43" t="str">
+      <c r="B44" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DATABASES : 'DATABASES' ;</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
-      <c r="A44" t="s">
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
         <v>583</v>
       </c>
-      <c r="B44" s="3" t="str">
+      <c r="B45" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DAY : 'DAY' ;</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
-      <c r="A45" t="s">
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
         <v>364</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B46" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DAY_HOUR : 'DAY_HOUR' ;</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
-      <c r="A46" t="s">
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
         <v>365</v>
       </c>
-      <c r="B46" t="str">
+      <c r="B47" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DAY_MICROSECOND : 'DAY_MICROSECOND' ;</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
-      <c r="A47" t="s">
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
         <v>366</v>
       </c>
-      <c r="B47" t="str">
+      <c r="B48" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DAY_MINUTE : 'DAY_MINUTE' ;</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
-      <c r="A48" t="s">
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
         <v>367</v>
       </c>
-      <c r="B48" t="str">
+      <c r="B49" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DAY_SECOND : 'DAY_SECOND' ;</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
         <v>368</v>
       </c>
-      <c r="B49" t="str">
+      <c r="B50" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DEC : 'DEC' ;</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
         <v>369</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B51" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DECIMAL : 'DECIMAL' ;</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
         <v>370</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B52" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DECLARE : 'DECLARE' ;</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
         <v>17</v>
       </c>
-      <c r="B52" t="str">
+      <c r="B53" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DEFAULT : 'DEFAULT' ;</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
         <v>371</v>
       </c>
-      <c r="B53" t="str">
+      <c r="B54" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DELAYED : 'DELAYED' ;</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
         <v>372</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B55" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DELETE : 'DELETE' ;</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
         <v>373</v>
       </c>
-      <c r="B55" t="str">
+      <c r="B56" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DELETE_DOMAIN_ID : 'DELETE_DOMAIN_ID' ;</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
         <v>374</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B57" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DESC : 'DESC' ;</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
         <v>375</v>
       </c>
-      <c r="B57" t="str">
+      <c r="B58" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DESCRIBE : 'DESCRIBE' ;</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
         <v>376</v>
       </c>
-      <c r="B58" t="str">
+      <c r="B59" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DETERMINISTIC : 'DETERMINISTIC' ;</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
         <v>377</v>
       </c>
-      <c r="B59" t="str">
+      <c r="B60" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DISTINCT : 'DISTINCT' ;</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
-      <c r="A60" t="s">
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
         <v>378</v>
       </c>
-      <c r="B60" t="str">
+      <c r="B61" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DISTINCTROW : 'DISTINCTROW' ;</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
-      <c r="A61" t="s">
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
         <v>379</v>
       </c>
-      <c r="B61" t="str">
+      <c r="B62" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DIV : 'DIV' ;</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
-      <c r="A62" t="s">
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
         <v>380</v>
       </c>
-      <c r="B62" t="str">
+      <c r="B63" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DO_DOMAIN_IDS : 'DO_DOMAIN_IDS' ;</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
-      <c r="A63" t="s">
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
         <v>381</v>
       </c>
-      <c r="B63" t="str">
+      <c r="B64" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DOUBLE : 'DOUBLE' ;</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
-      <c r="A64" t="s">
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
         <v>382</v>
       </c>
-      <c r="B64" t="str">
+      <c r="B65" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DROP : 'DROP' ;</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
-      <c r="A65" t="s">
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
         <v>383</v>
       </c>
-      <c r="B65" t="str">
+      <c r="B66" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>DUAL : 'DUAL' ;</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
-      <c r="A66" t="s">
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
         <v>384</v>
       </c>
-      <c r="B66" t="str">
+      <c r="B67" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EACH : 'EACH' ;</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
-      <c r="A67" t="s">
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
         <v>385</v>
       </c>
-      <c r="B67" t="str">
+      <c r="B68" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ELSE : 'ELSE' ;</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
-      <c r="A68" t="s">
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
         <v>386</v>
       </c>
-      <c r="B68" t="str">
+      <c r="B69" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ELSEIF : 'ELSEIF' ;</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
-      <c r="A69" t="s">
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
         <v>387</v>
       </c>
-      <c r="B69" t="str">
+      <c r="B70" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ENCLOSED : 'ENCLOSED' ;</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
-      <c r="A70" t="s">
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
         <v>388</v>
       </c>
-      <c r="B70" t="str">
+      <c r="B71" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ESCAPED : 'ESCAPED' ;</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
-      <c r="A71" t="s">
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
         <v>389</v>
       </c>
-      <c r="B71" t="str">
+      <c r="B72" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EXCEPT : 'EXCEPT' ;</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
-      <c r="A72" t="s">
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
         <v>390</v>
       </c>
-      <c r="B72" t="str">
+      <c r="B73" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EXISTS : 'EXISTS' ;</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
-      <c r="A73" t="s">
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
         <v>391</v>
       </c>
-      <c r="B73" t="str">
+      <c r="B74" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EXIT : 'EXIT' ;</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
-      <c r="A74" t="s">
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
         <v>581</v>
       </c>
-      <c r="B74" s="3" t="str">
+      <c r="B75" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EXPIRE : 'EXPIRE' ;</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
-      <c r="A75" t="s">
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
         <v>392</v>
       </c>
-      <c r="B75" t="str">
+      <c r="B76" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>EXPLAIN : 'EXPLAIN' ;</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="2" t="s">
+    <row r="77" spans="1:2">
+      <c r="A77" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="B76" t="str">
+      <c r="B77" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FALSE : 'FALSE' ;</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
-      <c r="A77" t="s">
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
         <v>393</v>
       </c>
-      <c r="B77" t="str">
+      <c r="B78" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FETCH : 'FETCH' ;</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
-      <c r="A78" t="s">
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
         <v>394</v>
       </c>
-      <c r="B78" t="str">
+      <c r="B79" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FLOAT : 'FLOAT' ;</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
-      <c r="A79" t="s">
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
         <v>395</v>
       </c>
-      <c r="B79" t="str">
+      <c r="B80" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FLOAT4 : 'FLOAT4' ;</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
-      <c r="A80" t="s">
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
         <v>396</v>
       </c>
-      <c r="B80" t="str">
+      <c r="B81" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FLOAT8 : 'FLOAT8' ;</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
-      <c r="A81" t="s">
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
         <v>397</v>
       </c>
-      <c r="B81" t="str">
+      <c r="B82" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FOR : 'FOR' ;</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
-      <c r="A82" t="s">
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
         <v>398</v>
       </c>
-      <c r="B82" t="str">
+      <c r="B83" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FORCE : 'FORCE' ;</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
-      <c r="A83" t="s">
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
         <v>399</v>
       </c>
-      <c r="B83" t="str">
+      <c r="B84" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FOREIGN : 'FOREIGN' ;</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
-      <c r="A84" t="s">
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
         <v>400</v>
       </c>
-      <c r="B84" t="str">
+      <c r="B85" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FROM : 'FROM' ;</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
-      <c r="A85" t="s">
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
         <v>401</v>
       </c>
-      <c r="B85" t="str">
+      <c r="B86" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>FULLTEXT : 'FULLTEXT' ;</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
-      <c r="A86" t="s">
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
         <v>402</v>
       </c>
-      <c r="B86" t="str">
+      <c r="B87" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>GENERAL : 'GENERAL' ;</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
-      <c r="A87" t="s">
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
         <v>403</v>
       </c>
-      <c r="B87" t="str">
+      <c r="B88" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>GRANT : 'GRANT' ;</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
-      <c r="A88" t="s">
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
         <v>80</v>
       </c>
-      <c r="B88" t="str">
+      <c r="B89" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>GROUP : 'GROUP' ;</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
-      <c r="A89" t="s">
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
         <v>404</v>
       </c>
-      <c r="B89" t="str">
+      <c r="B90" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>HAVING : 'HAVING' ;</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
-      <c r="A90" t="s">
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
         <v>405</v>
       </c>
-      <c r="B90" t="str">
+      <c r="B91" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>HIGH_PRIORITY : 'HIGH_PRIORITY' ;</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
-      <c r="A91" t="s">
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
         <v>406</v>
       </c>
-      <c r="B91" t="str">
+      <c r="B92" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>HOUR_MICROSECOND : 'HOUR_MICROSECOND' ;</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
-      <c r="A92" t="s">
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
         <v>407</v>
       </c>
-      <c r="B92" t="str">
+      <c r="B93" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>HOUR_MINUTE : 'HOUR_MINUTE' ;</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
-      <c r="A93" t="s">
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
         <v>408</v>
       </c>
-      <c r="B93" t="str">
+      <c r="B94" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>HOUR_SECOND : 'HOUR_SECOND' ;</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
-      <c r="A94" t="s">
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
         <v>571</v>
       </c>
-      <c r="B94" s="3" t="str">
+      <c r="B95" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IDENTIFIED : 'IDENTIFIED' ;</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
-      <c r="A95" t="s">
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
         <v>409</v>
       </c>
-      <c r="B95" t="str">
+      <c r="B96" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IF : 'IF' ;</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
-      <c r="A96" t="s">
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
         <v>410</v>
       </c>
-      <c r="B96" t="str">
+      <c r="B97" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IGNORE : 'IGNORE' ;</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
-      <c r="A97" t="s">
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
         <v>411</v>
       </c>
-      <c r="B97" t="str">
+      <c r="B98" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IGNORE_DOMAIN_IDS : 'IGNORE_DOMAIN_IDS' ;</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
-      <c r="A98" t="s">
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
         <v>412</v>
       </c>
-      <c r="B98" t="str">
+      <c r="B99" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IGNORE_SERVER_IDS : 'IGNORE_SERVER_IDS' ;</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
-      <c r="A99" t="s">
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
         <v>413</v>
       </c>
-      <c r="B99" t="str">
+      <c r="B100" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IN : 'IN' ;</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
-      <c r="A100" t="s">
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
         <v>33</v>
       </c>
-      <c r="B100" t="str">
+      <c r="B101" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INDEX : 'INDEX' ;</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
-      <c r="A101" t="s">
+    <row r="102" spans="1:2">
+      <c r="A102" t="s">
         <v>414</v>
       </c>
-      <c r="B101" t="str">
+      <c r="B102" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INFILE : 'INFILE' ;</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
-      <c r="A102" t="s">
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
         <v>415</v>
       </c>
-      <c r="B102" t="str">
+      <c r="B103" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INNER : 'INNER' ;</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
-      <c r="A103" t="s">
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
         <v>416</v>
       </c>
-      <c r="B103" t="str">
+      <c r="B104" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INOUT : 'INOUT' ;</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
-      <c r="A104" t="s">
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
         <v>417</v>
       </c>
-      <c r="B104" t="str">
+      <c r="B105" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INSENSITIVE : 'INSENSITIVE' ;</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
-      <c r="A105" t="s">
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
         <v>418</v>
       </c>
-      <c r="B105" t="str">
+      <c r="B106" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INSERT : 'INSERT' ;</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
-      <c r="A106" t="s">
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
         <v>419</v>
       </c>
-      <c r="B106" t="str">
+      <c r="B107" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT : 'INT' ;</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
-      <c r="A107" t="s">
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
         <v>420</v>
       </c>
-      <c r="B107" t="str">
+      <c r="B108" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT1 : 'INT1' ;</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
-      <c r="A108" t="s">
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
         <v>421</v>
       </c>
-      <c r="B108" t="str">
+      <c r="B109" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT2 : 'INT2' ;</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
-      <c r="A109" t="s">
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
         <v>422</v>
       </c>
-      <c r="B109" t="str">
+      <c r="B110" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT3 : 'INT3' ;</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
-      <c r="A110" t="s">
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
         <v>423</v>
       </c>
-      <c r="B110" t="str">
+      <c r="B111" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT4 : 'INT4' ;</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
-      <c r="A111" t="s">
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
         <v>424</v>
       </c>
-      <c r="B111" t="str">
+      <c r="B112" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INT8 : 'INT8' ;</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
-      <c r="A112" t="s">
+    <row r="113" spans="1:2">
+      <c r="A113" t="s">
         <v>425</v>
       </c>
-      <c r="B112" t="str">
+      <c r="B113" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INTEGER : 'INTEGER' ;</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
-      <c r="A113" t="s">
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
         <v>426</v>
       </c>
-      <c r="B113" t="str">
+      <c r="B114" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INTERSECT : 'INTERSECT' ;</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
-      <c r="A114" t="s">
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
         <v>427</v>
       </c>
-      <c r="B114" t="str">
+      <c r="B115" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INTERVAL : 'INTERVAL' ;</v>
       </c>
     </row>
-    <row r="115" spans="1:2">
-      <c r="A115" t="s">
+    <row r="116" spans="1:2">
+      <c r="A116" t="s">
         <v>428</v>
       </c>
-      <c r="B115" t="str">
+      <c r="B116" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>INTO : 'INTO' ;</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
-      <c r="A116" t="s">
+    <row r="117" spans="1:2">
+      <c r="A117" t="s">
         <v>429</v>
       </c>
-      <c r="B116" t="str">
+      <c r="B117" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>IS : 'IS' ;</v>
       </c>
     </row>
-    <row r="117" spans="1:2">
-      <c r="A117" t="s">
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
         <v>574</v>
       </c>
-      <c r="B117" s="3" t="str">
+      <c r="B118" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ISSUER : 'ISSUER' ;</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
-      <c r="A118" t="s">
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
         <v>430</v>
       </c>
-      <c r="B118" t="str">
+      <c r="B119" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ITERATE : 'ITERATE' ;</v>
       </c>
     </row>
-    <row r="119" spans="1:2">
-      <c r="A119" t="s">
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
         <v>431</v>
       </c>
-      <c r="B119" t="str">
+      <c r="B120" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>JOIN : 'JOIN' ;</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
-      <c r="A120" t="s">
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
         <v>313</v>
       </c>
-      <c r="B120" t="str">
+      <c r="B121" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>KEY : 'KEY' ;</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
-      <c r="A121" t="s">
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
         <v>432</v>
       </c>
-      <c r="B121" t="str">
+      <c r="B122" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>KEYS : 'KEYS' ;</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
-      <c r="A122" t="s">
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
         <v>433</v>
       </c>
-      <c r="B122" t="str">
+      <c r="B123" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>KILL : 'KILL' ;</v>
       </c>
     </row>
-    <row r="123" spans="1:2">
-      <c r="A123" t="s">
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
         <v>434</v>
       </c>
-      <c r="B123" t="str">
+      <c r="B124" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LEADING : 'LEADING' ;</v>
       </c>
     </row>
-    <row r="124" spans="1:2">
-      <c r="A124" t="s">
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
         <v>435</v>
       </c>
-      <c r="B124" t="str">
+      <c r="B125" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LEAVE : 'LEAVE' ;</v>
       </c>
     </row>
-    <row r="125" spans="1:2">
-      <c r="A125" t="s">
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
         <v>436</v>
       </c>
-      <c r="B125" t="str">
+      <c r="B126" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LEFT : 'LEFT' ;</v>
       </c>
     </row>
-    <row r="126" spans="1:2">
-      <c r="A126" t="s">
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
         <v>437</v>
       </c>
-      <c r="B126" t="str">
+      <c r="B127" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LIKE : 'LIKE' ;</v>
       </c>
     </row>
-    <row r="127" spans="1:2">
-      <c r="A127" t="s">
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
         <v>438</v>
       </c>
-      <c r="B127" t="str">
+      <c r="B128" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LIMIT : 'LIMIT' ;</v>
       </c>
     </row>
-    <row r="128" spans="1:2">
-      <c r="A128" t="s">
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
         <v>439</v>
       </c>
-      <c r="B128" t="str">
+      <c r="B129" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LINEAR : 'LINEAR' ;</v>
       </c>
     </row>
-    <row r="129" spans="1:2">
-      <c r="A129" t="s">
+    <row r="130" spans="1:2">
+      <c r="A130" t="s">
         <v>440</v>
       </c>
-      <c r="B129" t="str">
+      <c r="B130" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LINES : 'LINES' ;</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
-      <c r="A130" t="s">
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
         <v>441</v>
       </c>
-      <c r="B130" t="str">
+      <c r="B131" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOAD : 'LOAD' ;</v>
       </c>
     </row>
-    <row r="131" spans="1:2">
-      <c r="A131" t="s">
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
         <v>442</v>
       </c>
-      <c r="B131" t="str">
+      <c r="B132" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOCALTIME : 'LOCALTIME' ;</v>
       </c>
     </row>
-    <row r="132" spans="1:2">
-      <c r="A132" t="s">
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
         <v>443</v>
       </c>
-      <c r="B132" t="str">
+      <c r="B133" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOCALTIMESTAMP : 'LOCALTIMESTAMP' ;</v>
       </c>
     </row>
-    <row r="133" spans="1:2">
-      <c r="A133" t="s">
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
         <v>444</v>
       </c>
-      <c r="B133" t="str">
+      <c r="B134" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOCK : 'LOCK' ;</v>
       </c>
     </row>
-    <row r="134" spans="1:2">
-      <c r="A134" t="s">
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
         <v>445</v>
       </c>
-      <c r="B134" t="str">
+      <c r="B135" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LONG : 'LONG' ;</v>
       </c>
     </row>
-    <row r="135" spans="1:2">
-      <c r="A135" t="s">
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
         <v>446</v>
       </c>
-      <c r="B135" t="str">
+      <c r="B136" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LONGBLOB : 'LONGBLOB' ;</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
-      <c r="A136" t="s">
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
         <v>447</v>
       </c>
-      <c r="B136" t="str">
+      <c r="B137" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LONGTEXT : 'LONGTEXT' ;</v>
       </c>
     </row>
-    <row r="137" spans="1:2">
-      <c r="A137" t="s">
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
         <v>448</v>
       </c>
-      <c r="B137" t="str">
+      <c r="B138" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOOP : 'LOOP' ;</v>
       </c>
     </row>
-    <row r="138" spans="1:2">
-      <c r="A138" t="s">
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
         <v>449</v>
       </c>
-      <c r="B138" t="str">
+      <c r="B139" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>LOW_PRIORITY : 'LOW_PRIORITY' ;</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
-      <c r="A139" t="s">
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
         <v>450</v>
       </c>
-      <c r="B139" t="str">
+      <c r="B140" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MASTER_HEARTBEAT_PERIOD : 'MASTER_HEARTBEAT_PERIOD' ;</v>
       </c>
     </row>
-    <row r="140" spans="1:2">
-      <c r="A140" t="s">
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
         <v>451</v>
       </c>
-      <c r="B140" t="str">
+      <c r="B141" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MASTER_SSL_VERIFY_SERVER_CERT : 'MASTER_SSL_VERIFY_SERVER_CERT' ;</v>
       </c>
     </row>
-    <row r="141" spans="1:2">
-      <c r="A141" t="s">
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
         <v>452</v>
       </c>
-      <c r="B141" t="str">
+      <c r="B142" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MATCH : 'MATCH' ;</v>
       </c>
     </row>
-    <row r="142" spans="1:2">
-      <c r="A142" t="s">
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
         <v>578</v>
       </c>
-      <c r="B142" s="3" t="str">
+      <c r="B143" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAX_CONNECTIONS_PER_HOUR : 'MAX_CONNECTIONS_PER_HOUR' ;</v>
       </c>
     </row>
-    <row r="143" spans="1:2">
-      <c r="A143" t="s">
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
         <v>576</v>
       </c>
-      <c r="B143" s="3" t="str">
+      <c r="B144" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAX_QUERIES_PER_HOUR : 'MAX_QUERIES_PER_HOUR' ;</v>
       </c>
     </row>
-    <row r="144" spans="1:2">
-      <c r="A144" t="s">
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
         <v>580</v>
       </c>
-      <c r="B144" s="3" t="str">
+      <c r="B145" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAX_STATEMENT_TIME : 'MAX_STATEMENT_TIME' ;</v>
       </c>
     </row>
-    <row r="145" spans="1:2">
-      <c r="A145" t="s">
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
         <v>577</v>
       </c>
-      <c r="B145" s="3" t="str">
+      <c r="B146" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAX_UPDATES_PER_HOUR : 'MAX_UPDATES_PER_HOUR' ;</v>
       </c>
     </row>
-    <row r="146" spans="1:2">
-      <c r="A146" t="s">
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
         <v>579</v>
       </c>
-      <c r="B146" s="3" t="str">
+      <c r="B147" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAX_USER_CONNECTIONS : 'MAX_USER_CONNECTIONS' ;</v>
       </c>
     </row>
-    <row r="147" spans="1:2">
-      <c r="A147" t="s">
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
         <v>453</v>
       </c>
-      <c r="B147" t="str">
+      <c r="B148" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MAXVALUE : 'MAXVALUE' ;</v>
       </c>
     </row>
-    <row r="148" spans="1:2">
-      <c r="A148" t="s">
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
         <v>454</v>
       </c>
-      <c r="B148" t="str">
+      <c r="B149" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MEDIUMBLOB : 'MEDIUMBLOB' ;</v>
       </c>
     </row>
-    <row r="149" spans="1:2">
-      <c r="A149" t="s">
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
         <v>455</v>
       </c>
-      <c r="B149" t="str">
+      <c r="B150" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MEDIUMINT : 'MEDIUMINT' ;</v>
       </c>
     </row>
-    <row r="150" spans="1:2">
-      <c r="A150" t="s">
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
         <v>456</v>
       </c>
-      <c r="B150" t="str">
+      <c r="B151" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MEDIUMTEXT : 'MEDIUMTEXT' ;</v>
       </c>
     </row>
-    <row r="151" spans="1:2">
-      <c r="A151" t="s">
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
         <v>457</v>
       </c>
-      <c r="B151" t="str">
+      <c r="B152" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MIDDLEINT : 'MIDDLEINT' ;</v>
       </c>
     </row>
-    <row r="152" spans="1:2">
-      <c r="A152" t="s">
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
         <v>458</v>
       </c>
-      <c r="B152" t="str">
+      <c r="B153" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MINUTE_MICROSECOND : 'MINUTE_MICROSECOND' ;</v>
       </c>
     </row>
-    <row r="153" spans="1:2">
-      <c r="A153" t="s">
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
         <v>459</v>
       </c>
-      <c r="B153" t="str">
+      <c r="B154" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MINUTE_SECOND : 'MINUTE_SECOND' ;</v>
       </c>
     </row>
-    <row r="154" spans="1:2">
-      <c r="A154" t="s">
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
         <v>460</v>
       </c>
-      <c r="B154" t="str">
+      <c r="B155" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MOD : 'MOD' ;</v>
       </c>
     </row>
-    <row r="155" spans="1:2">
-      <c r="A155" t="s">
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
         <v>461</v>
       </c>
-      <c r="B155" t="str">
+      <c r="B156" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>MODIFIES : 'MODIFIES' ;</v>
       </c>
     </row>
-    <row r="156" spans="1:2">
-      <c r="A156" t="s">
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
         <v>462</v>
       </c>
-      <c r="B156" t="str">
+      <c r="B157" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NATURAL : 'NATURAL' ;</v>
       </c>
     </row>
-    <row r="157" spans="1:2">
-      <c r="A157" t="s">
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
         <v>582</v>
       </c>
-      <c r="B157" s="3" t="str">
+      <c r="B158" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NEVER : 'NEVER' ;</v>
       </c>
     </row>
-    <row r="158" spans="1:2">
-      <c r="A158" t="s">
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
         <v>464</v>
       </c>
-      <c r="B158" t="str">
+      <c r="B159" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NO_WRITE_TO_BINLOG : 'NO_WRITE_TO_BINLOG' ;</v>
       </c>
     </row>
-    <row r="159" spans="1:2">
-      <c r="A159" t="s">
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>586</v>
+      </c>
+      <c r="B160" s="3" t="str">
+        <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
+        <v>NONE : 'NONE' ;</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
         <v>463</v>
       </c>
-      <c r="B159" t="str">
+      <c r="B161" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NOT : 'NOT' ;</v>
       </c>
     </row>
-    <row r="160" spans="1:2">
-      <c r="A160" t="s">
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
         <v>465</v>
       </c>
-      <c r="B160" t="str">
+      <c r="B162" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NULL : 'NULL' ;</v>
       </c>
     </row>
-    <row r="161" spans="1:2">
-      <c r="A161" t="s">
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
         <v>466</v>
       </c>
-      <c r="B161" t="str">
+      <c r="B163" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>NUMERIC : 'NUMERIC' ;</v>
       </c>
     </row>
-    <row r="162" spans="1:2">
-      <c r="A162" t="s">
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
         <v>566</v>
       </c>
-      <c r="B162" t="str">
+      <c r="B164" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OFFSET : 'OFFSET' ;</v>
       </c>
     </row>
-    <row r="163" spans="1:2">
-      <c r="A163" t="s">
+    <row r="165" spans="1:2" ht="15">
+      <c r="A165" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="B165" s="3" t="str">
+        <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
+        <v>OLD_PASSWORD : 'OLD_PASSWORD' ;</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" t="s">
         <v>467</v>
       </c>
-      <c r="B163" t="str">
+      <c r="B166" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ON : 'ON' ;</v>
       </c>
     </row>
-    <row r="164" spans="1:2">
-      <c r="A164" t="s">
+    <row r="167" spans="1:2">
+      <c r="A167" t="s">
         <v>468</v>
       </c>
-      <c r="B164" t="str">
+      <c r="B167" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OPTIMIZE : 'OPTIMIZE' ;</v>
       </c>
     </row>
-    <row r="165" spans="1:2">
-      <c r="A165" t="s">
+    <row r="168" spans="1:2">
+      <c r="A168" t="s">
         <v>469</v>
       </c>
-      <c r="B165" t="str">
+      <c r="B168" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OPTION : 'OPTION' ;</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
-      <c r="A166" t="s">
+    <row r="169" spans="1:2">
+      <c r="A169" t="s">
         <v>470</v>
       </c>
-      <c r="B166" t="str">
+      <c r="B169" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OPTIONALLY : 'OPTIONALLY' ;</v>
       </c>
     </row>
-    <row r="167" spans="1:2">
-      <c r="A167" t="s">
+    <row r="170" spans="1:2">
+      <c r="A170" t="s">
         <v>471</v>
       </c>
-      <c r="B167" t="str">
+      <c r="B170" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OR : 'OR' ;</v>
       </c>
     </row>
-    <row r="168" spans="1:2">
-      <c r="A168" t="s">
+    <row r="171" spans="1:2">
+      <c r="A171" t="s">
         <v>472</v>
       </c>
-      <c r="B168" t="str">
+      <c r="B171" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ORDER : 'ORDER' ;</v>
       </c>
     </row>
-    <row r="169" spans="1:2">
-      <c r="A169" t="s">
+    <row r="172" spans="1:2">
+      <c r="A172" t="s">
         <v>473</v>
       </c>
-      <c r="B169" t="str">
+      <c r="B172" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OUT : 'OUT' ;</v>
       </c>
     </row>
-    <row r="170" spans="1:2">
-      <c r="A170" t="s">
+    <row r="173" spans="1:2">
+      <c r="A173" t="s">
         <v>474</v>
       </c>
-      <c r="B170" t="str">
+      <c r="B173" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OUTER : 'OUTER' ;</v>
       </c>
     </row>
-    <row r="171" spans="1:2">
-      <c r="A171" t="s">
+    <row r="174" spans="1:2">
+      <c r="A174" t="s">
         <v>475</v>
       </c>
-      <c r="B171" t="str">
+      <c r="B174" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OUTFILE : 'OUTFILE' ;</v>
       </c>
     </row>
-    <row r="172" spans="1:2">
-      <c r="A172" t="s">
+    <row r="175" spans="1:2">
+      <c r="A175" t="s">
         <v>476</v>
       </c>
-      <c r="B172" t="str">
+      <c r="B175" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>OVER : 'OVER' ;</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
-      <c r="A173" t="s">
+    <row r="176" spans="1:2">
+      <c r="A176" t="s">
         <v>477</v>
       </c>
-      <c r="B173" t="str">
+      <c r="B176" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PAGE_CHECKSUM : 'PAGE_CHECKSUM' ;</v>
       </c>
     </row>
-    <row r="174" spans="1:2">
-      <c r="A174" t="s">
+    <row r="177" spans="1:2">
+      <c r="A177" t="s">
         <v>478</v>
       </c>
-      <c r="B174" t="str">
+      <c r="B177" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PARSE_VCOL_EXPR : 'PARSE_VCOL_EXPR' ;</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
-      <c r="A175" t="s">
+    <row r="178" spans="1:2">
+      <c r="A178" t="s">
         <v>479</v>
       </c>
-      <c r="B175" t="str">
+      <c r="B178" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PARTITION : 'PARTITION' ;</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
-      <c r="A176" t="s">
+    <row r="179" spans="1:2">
+      <c r="A179" t="s">
         <v>570</v>
       </c>
-      <c r="B176" s="3" t="str">
+      <c r="B179" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PASSWORD : 'PASSWORD' ;</v>
       </c>
     </row>
-    <row r="177" spans="1:2">
-      <c r="A177" t="s">
+    <row r="180" spans="1:2">
+      <c r="A180" t="s">
         <v>480</v>
       </c>
-      <c r="B177" t="str">
+      <c r="B180" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PRECISION : 'PRECISION' ;</v>
       </c>
     </row>
-    <row r="178" spans="1:2">
-      <c r="A178" t="s">
+    <row r="181" spans="1:2">
+      <c r="A181" t="s">
         <v>481</v>
       </c>
-      <c r="B178" t="str">
+      <c r="B181" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PRIMARY : 'PRIMARY' ;</v>
       </c>
     </row>
-    <row r="179" spans="1:2">
-      <c r="A179" t="s">
+    <row r="182" spans="1:2">
+      <c r="A182" t="s">
         <v>40</v>
       </c>
-      <c r="B179" t="str">
+      <c r="B182" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PROCEDURE : 'PROCEDURE' ;</v>
       </c>
     </row>
-    <row r="180" spans="1:2">
-      <c r="A180" t="s">
+    <row r="183" spans="1:2">
+      <c r="A183" t="s">
         <v>482</v>
       </c>
-      <c r="B180" t="str">
+      <c r="B183" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>PURGE : 'PURGE' ;</v>
       </c>
     </row>
-    <row r="181" spans="1:2">
-      <c r="A181" t="s">
+    <row r="184" spans="1:2">
+      <c r="A184" t="s">
         <v>483</v>
       </c>
-      <c r="B181" t="str">
+      <c r="B184" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RANGE : 'RANGE' ;</v>
       </c>
     </row>
-    <row r="182" spans="1:2">
-      <c r="A182" t="s">
+    <row r="185" spans="1:2">
+      <c r="A185" t="s">
         <v>484</v>
       </c>
-      <c r="B182" t="str">
+      <c r="B185" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>READ : 'READ' ;</v>
       </c>
     </row>
-    <row r="183" spans="1:2">
-      <c r="A183" t="s">
+    <row r="186" spans="1:2">
+      <c r="A186" t="s">
         <v>486</v>
       </c>
-      <c r="B183" t="str">
+      <c r="B186" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>READ_WRITE : 'READ_WRITE' ;</v>
       </c>
     </row>
-    <row r="184" spans="1:2">
-      <c r="A184" t="s">
+    <row r="187" spans="1:2">
+      <c r="A187" t="s">
         <v>485</v>
       </c>
-      <c r="B184" t="str">
+      <c r="B187" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>READS : 'READS' ;</v>
       </c>
     </row>
-    <row r="185" spans="1:2">
-      <c r="A185" t="s">
+    <row r="188" spans="1:2">
+      <c r="A188" t="s">
         <v>487</v>
       </c>
-      <c r="B185" t="str">
+      <c r="B188" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REAL : 'REAL' ;</v>
       </c>
     </row>
-    <row r="186" spans="1:2">
-      <c r="A186" t="s">
+    <row r="189" spans="1:2">
+      <c r="A189" t="s">
         <v>488</v>
       </c>
-      <c r="B186" t="str">
+      <c r="B189" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RECURSIVE : 'RECURSIVE' ;</v>
       </c>
     </row>
-    <row r="187" spans="1:2">
-      <c r="A187" t="s">
+    <row r="190" spans="1:2">
+      <c r="A190" t="s">
         <v>489</v>
       </c>
-      <c r="B187" t="str">
+      <c r="B190" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REF_SYSTEM_ID : 'REF_SYSTEM_ID' ;</v>
       </c>
     </row>
-    <row r="188" spans="1:2">
-      <c r="A188" t="s">
+    <row r="191" spans="1:2">
+      <c r="A191" t="s">
         <v>490</v>
       </c>
-      <c r="B188" t="str">
+      <c r="B191" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REFERENCES : 'REFERENCES' ;</v>
       </c>
     </row>
-    <row r="189" spans="1:2">
-      <c r="A189" t="s">
+    <row r="192" spans="1:2">
+      <c r="A192" t="s">
         <v>491</v>
       </c>
-      <c r="B189" t="str">
+      <c r="B192" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REGEXP : 'REGEXP' ;</v>
       </c>
     </row>
-    <row r="190" spans="1:2">
-      <c r="A190" t="s">
+    <row r="193" spans="1:2">
+      <c r="A193" t="s">
         <v>492</v>
       </c>
-      <c r="B190" t="str">
+      <c r="B193" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RELEASE : 'RELEASE' ;</v>
       </c>
     </row>
-    <row r="191" spans="1:2">
-      <c r="A191" t="s">
+    <row r="194" spans="1:2">
+      <c r="A194" t="s">
         <v>493</v>
       </c>
-      <c r="B191" t="str">
+      <c r="B194" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RENAME : 'RENAME' ;</v>
       </c>
     </row>
-    <row r="192" spans="1:2">
-      <c r="A192" t="s">
+    <row r="195" spans="1:2">
+      <c r="A195" t="s">
         <v>494</v>
       </c>
-      <c r="B192" t="str">
+      <c r="B195" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REPEAT : 'REPEAT' ;</v>
       </c>
     </row>
-    <row r="193" spans="1:2">
-      <c r="A193" t="s">
+    <row r="196" spans="1:2">
+      <c r="A196" t="s">
         <v>495</v>
       </c>
-      <c r="B193" t="str">
+      <c r="B196" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REPLACE : 'REPLACE' ;</v>
       </c>
     </row>
-    <row r="194" spans="1:2">
-      <c r="A194" t="s">
+    <row r="197" spans="1:2">
+      <c r="A197" t="s">
         <v>496</v>
       </c>
-      <c r="B194" t="str">
+      <c r="B197" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REQUIRE : 'REQUIRE' ;</v>
       </c>
     </row>
-    <row r="195" spans="1:2">
-      <c r="A195" t="s">
+    <row r="198" spans="1:2">
+      <c r="A198" t="s">
         <v>497</v>
       </c>
-      <c r="B195" t="str">
+      <c r="B198" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RESIGNAL : 'RESIGNAL' ;</v>
       </c>
     </row>
-    <row r="196" spans="1:2">
-      <c r="A196" t="s">
+    <row r="199" spans="1:2">
+      <c r="A199" t="s">
         <v>498</v>
       </c>
-      <c r="B196" t="str">
+      <c r="B199" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RESTRICT : 'RESTRICT' ;</v>
       </c>
     </row>
-    <row r="197" spans="1:2">
-      <c r="A197" t="s">
+    <row r="200" spans="1:2">
+      <c r="A200" t="s">
         <v>499</v>
       </c>
-      <c r="B197" t="str">
+      <c r="B200" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RETURN : 'RETURN' ;</v>
       </c>
     </row>
-    <row r="198" spans="1:2">
-      <c r="A198" t="s">
+    <row r="201" spans="1:2">
+      <c r="A201" t="s">
         <v>500</v>
       </c>
-      <c r="B198" t="str">
+      <c r="B201" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RETURNING : 'RETURNING' ;</v>
       </c>
     </row>
-    <row r="199" spans="1:2">
-      <c r="A199" t="s">
+    <row r="202" spans="1:2">
+      <c r="A202" t="s">
         <v>501</v>
       </c>
-      <c r="B199" t="str">
+      <c r="B202" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>REVOKE : 'REVOKE' ;</v>
       </c>
     </row>
-    <row r="200" spans="1:2">
-      <c r="A200" t="s">
+    <row r="203" spans="1:2">
+      <c r="A203" t="s">
         <v>502</v>
       </c>
-      <c r="B200" t="str">
+      <c r="B203" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RIGHT : 'RIGHT' ;</v>
       </c>
     </row>
-    <row r="201" spans="1:2">
-      <c r="A201" t="s">
+    <row r="204" spans="1:2">
+      <c r="A204" t="s">
         <v>503</v>
       </c>
-      <c r="B201" t="str">
+      <c r="B204" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>RLIKE : 'RLIKE' ;</v>
       </c>
     </row>
-    <row r="202" spans="1:2">
-      <c r="A202" t="s">
+    <row r="205" spans="1:2">
+      <c r="A205" t="s">
         <v>44</v>
       </c>
-      <c r="B202" t="str">
+      <c r="B205" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ROLE : 'ROLE' ;</v>
       </c>
     </row>
-    <row r="203" spans="1:2">
-      <c r="A203" t="s">
+    <row r="206" spans="1:2">
+      <c r="A206" t="s">
         <v>567</v>
       </c>
-      <c r="B203" t="str">
+      <c r="B206" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ROW_NUMBER : 'ROW_NUMBER' ;</v>
       </c>
     </row>
-    <row r="204" spans="1:2">
-      <c r="A204" t="s">
+    <row r="207" spans="1:2">
+      <c r="A207" t="s">
         <v>504</v>
       </c>
-      <c r="B204" t="str">
+      <c r="B207" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ROWS : 'ROWS' ;</v>
       </c>
     </row>
-    <row r="205" spans="1:2">
-      <c r="A205" t="s">
+    <row r="208" spans="1:2">
+      <c r="A208" t="s">
         <v>47</v>
       </c>
-      <c r="B205" t="str">
+      <c r="B208" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SCHEMA : 'SCHEMA' ;</v>
       </c>
     </row>
-    <row r="206" spans="1:2">
-      <c r="A206" t="s">
+    <row r="209" spans="1:2">
+      <c r="A209" t="s">
         <v>505</v>
       </c>
-      <c r="B206" t="str">
+      <c r="B209" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SCHEMAS : 'SCHEMAS' ;</v>
       </c>
     </row>
-    <row r="207" spans="1:2">
-      <c r="A207" t="s">
+    <row r="210" spans="1:2">
+      <c r="A210" t="s">
         <v>506</v>
       </c>
-      <c r="B207" t="str">
+      <c r="B210" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SECOND_MICROSECOND : 'SECOND_MICROSECOND' ;</v>
       </c>
     </row>
-    <row r="208" spans="1:2">
-      <c r="A208" t="s">
+    <row r="211" spans="1:2">
+      <c r="A211" t="s">
         <v>507</v>
       </c>
-      <c r="B208" t="str">
+      <c r="B211" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SELECT : 'SELECT' ;</v>
       </c>
     </row>
-    <row r="209" spans="1:2">
-      <c r="A209" t="s">
+    <row r="212" spans="1:2">
+      <c r="A212" t="s">
         <v>508</v>
       </c>
-      <c r="B209" t="str">
+      <c r="B212" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SENSITIVE : 'SENSITIVE' ;</v>
       </c>
     </row>
-    <row r="210" spans="1:2">
-      <c r="A210" t="s">
+    <row r="213" spans="1:2">
+      <c r="A213" t="s">
         <v>509</v>
       </c>
-      <c r="B210" t="str">
+      <c r="B213" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SEPARATOR : 'SEPARATOR' ;</v>
       </c>
     </row>
-    <row r="211" spans="1:2">
-      <c r="A211" t="s">
+    <row r="214" spans="1:2">
+      <c r="A214" t="s">
+        <v>588</v>
+      </c>
+      <c r="B214" s="3" t="str">
+        <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
+        <v>SESSION : 'SESSION' ;</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" t="s">
         <v>510</v>
       </c>
-      <c r="B211" t="str">
+      <c r="B215" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SET : 'SET' ;</v>
       </c>
     </row>
-    <row r="212" spans="1:2">
-      <c r="A212" t="s">
+    <row r="216" spans="1:2">
+      <c r="A216" t="s">
         <v>511</v>
       </c>
-      <c r="B212" t="str">
+      <c r="B216" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SHOW : 'SHOW' ;</v>
       </c>
     </row>
-    <row r="213" spans="1:2">
-      <c r="A213" t="s">
+    <row r="217" spans="1:2">
+      <c r="A217" t="s">
         <v>512</v>
       </c>
-      <c r="B213" t="str">
+      <c r="B217" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SIGNAL : 'SIGNAL' ;</v>
       </c>
     </row>
-    <row r="214" spans="1:2">
-      <c r="A214" t="s">
+    <row r="218" spans="1:2">
+      <c r="A218" t="s">
         <v>513</v>
       </c>
-      <c r="B214" t="str">
+      <c r="B218" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SLOW : 'SLOW' ;</v>
       </c>
     </row>
-    <row r="215" spans="1:2">
-      <c r="A215" t="s">
+    <row r="219" spans="1:2">
+      <c r="A219" t="s">
         <v>514</v>
       </c>
-      <c r="B215" t="str">
+      <c r="B219" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SMALLINT : 'SMALLINT' ;</v>
       </c>
     </row>
-    <row r="216" spans="1:2">
-      <c r="A216" t="s">
+    <row r="220" spans="1:2">
+      <c r="A220" t="s">
         <v>515</v>
       </c>
-      <c r="B216" t="str">
+      <c r="B220" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SPATIAL : 'SPATIAL' ;</v>
       </c>
     </row>
-    <row r="217" spans="1:2">
-      <c r="A217" t="s">
+    <row r="221" spans="1:2">
+      <c r="A221" t="s">
         <v>516</v>
       </c>
-      <c r="B217" t="str">
+      <c r="B221" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SPECIFIC : 'SPECIFIC' ;</v>
       </c>
     </row>
-    <row r="218" spans="1:2">
-      <c r="A218" t="s">
+    <row r="222" spans="1:2">
+      <c r="A222" t="s">
         <v>517</v>
       </c>
-      <c r="B218" t="str">
+      <c r="B222" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQL : 'SQL' ;</v>
       </c>
     </row>
-    <row r="219" spans="1:2">
-      <c r="A219" t="s">
+    <row r="223" spans="1:2">
+      <c r="A223" t="s">
         <v>521</v>
       </c>
-      <c r="B219" t="str">
+      <c r="B223" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQL_BIG_RESULT : 'SQL_BIG_RESULT' ;</v>
       </c>
     </row>
-    <row r="220" spans="1:2">
-      <c r="A220" t="s">
+    <row r="224" spans="1:2">
+      <c r="A224" t="s">
         <v>522</v>
       </c>
-      <c r="B220" t="str">
+      <c r="B224" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQL_CALC_FOUND_ROWS : 'SQL_CALC_FOUND_ROWS' ;</v>
       </c>
     </row>
-    <row r="221" spans="1:2">
-      <c r="A221" t="s">
+    <row r="225" spans="1:2">
+      <c r="A225" t="s">
         <v>523</v>
       </c>
-      <c r="B221" t="str">
+      <c r="B225" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQL_SMALL_RESULT : 'SQL_SMALL_RESULT' ;</v>
       </c>
     </row>
-    <row r="222" spans="1:2">
-      <c r="A222" t="s">
+    <row r="226" spans="1:2">
+      <c r="A226" t="s">
         <v>518</v>
       </c>
-      <c r="B222" t="str">
+      <c r="B226" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQLEXCEPTION : 'SQLEXCEPTION' ;</v>
       </c>
     </row>
-    <row r="223" spans="1:2">
-      <c r="A223" t="s">
+    <row r="227" spans="1:2">
+      <c r="A227" t="s">
         <v>519</v>
       </c>
-      <c r="B223" t="str">
+      <c r="B227" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQLSTATE : 'SQLSTATE' ;</v>
       </c>
     </row>
-    <row r="224" spans="1:2">
-      <c r="A224" t="s">
+    <row r="228" spans="1:2">
+      <c r="A228" t="s">
         <v>520</v>
       </c>
-      <c r="B224" t="str">
+      <c r="B228" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SQLWARNING : 'SQLWARNING' ;</v>
       </c>
     </row>
-    <row r="225" spans="1:2">
-      <c r="A225" t="s">
+    <row r="229" spans="1:2">
+      <c r="A229" t="s">
         <v>524</v>
       </c>
-      <c r="B225" t="str">
+      <c r="B229" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SSL : 'SSL' ;</v>
       </c>
     </row>
-    <row r="226" spans="1:2">
-      <c r="A226" t="s">
+    <row r="230" spans="1:2">
+      <c r="A230" t="s">
         <v>525</v>
       </c>
-      <c r="B226" t="str">
+      <c r="B230" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>STARTING : 'STARTING' ;</v>
       </c>
     </row>
-    <row r="227" spans="1:2">
-      <c r="A227" t="s">
+    <row r="231" spans="1:2">
+      <c r="A231" t="s">
         <v>526</v>
       </c>
-      <c r="B227" t="str">
+      <c r="B231" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>STATS_AUTO_RECALC : 'STATS_AUTO_RECALC' ;</v>
       </c>
     </row>
-    <row r="228" spans="1:2">
-      <c r="A228" t="s">
+    <row r="232" spans="1:2">
+      <c r="A232" t="s">
         <v>527</v>
       </c>
-      <c r="B228" t="str">
+      <c r="B232" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>STATS_PERSISTENT : 'STATS_PERSISTENT' ;</v>
       </c>
     </row>
-    <row r="229" spans="1:2">
-      <c r="A229" t="s">
+    <row r="233" spans="1:2">
+      <c r="A233" t="s">
         <v>528</v>
       </c>
-      <c r="B229" t="str">
+      <c r="B233" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>STATS_SAMPLE_PAGES : 'STATS_SAMPLE_PAGES' ;</v>
       </c>
     </row>
-    <row r="230" spans="1:2">
-      <c r="A230" t="s">
+    <row r="234" spans="1:2">
+      <c r="A234" t="s">
         <v>529</v>
       </c>
-      <c r="B230" t="str">
+      <c r="B234" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>STRAIGHT_JOIN : 'STRAIGHT_JOIN' ;</v>
       </c>
     </row>
-    <row r="231" spans="1:2">
-      <c r="A231" t="s">
+    <row r="235" spans="1:2">
+      <c r="A235" t="s">
         <v>575</v>
       </c>
-      <c r="B231" s="3" t="str">
+      <c r="B235" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>SUBJECT : 'SUBJECT' ;</v>
       </c>
     </row>
-    <row r="232" spans="1:2">
-      <c r="A232" t="s">
+    <row r="236" spans="1:2">
+      <c r="A236" t="s">
         <v>60</v>
       </c>
-      <c r="B232" t="str">
+      <c r="B236" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TABLE : 'TABLE' ;</v>
       </c>
     </row>
-    <row r="233" spans="1:2">
-      <c r="A233" t="s">
+    <row r="237" spans="1:2">
+      <c r="A237" t="s">
         <v>530</v>
       </c>
-      <c r="B233" t="str">
+      <c r="B237" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TERMINATED : 'TERMINATED' ;</v>
       </c>
     </row>
-    <row r="234" spans="1:2">
-      <c r="A234" t="s">
+    <row r="238" spans="1:2">
+      <c r="A238" t="s">
         <v>531</v>
       </c>
-      <c r="B234" t="str">
+      <c r="B238" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>THEN : 'THEN' ;</v>
       </c>
     </row>
-    <row r="235" spans="1:2">
-      <c r="A235" t="s">
+    <row r="239" spans="1:2">
+      <c r="A239" t="s">
         <v>532</v>
       </c>
-      <c r="B235" t="str">
+      <c r="B239" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TINYBLOB : 'TINYBLOB' ;</v>
       </c>
     </row>
-    <row r="236" spans="1:2">
-      <c r="A236" t="s">
+    <row r="240" spans="1:2">
+      <c r="A240" t="s">
         <v>533</v>
       </c>
-      <c r="B236" t="str">
+      <c r="B240" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TINYINT : 'TINYINT' ;</v>
       </c>
     </row>
-    <row r="237" spans="1:2">
-      <c r="A237" t="s">
+    <row r="241" spans="1:2">
+      <c r="A241" t="s">
         <v>534</v>
       </c>
-      <c r="B237" t="str">
+      <c r="B241" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TINYTEXT : 'TINYTEXT' ;</v>
       </c>
     </row>
-    <row r="238" spans="1:2">
-      <c r="A238" t="s">
+    <row r="242" spans="1:2">
+      <c r="A242" t="s">
         <v>535</v>
       </c>
-      <c r="B238" t="str">
+      <c r="B242" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TO : 'TO' ;</v>
       </c>
     </row>
-    <row r="239" spans="1:2">
-      <c r="A239" t="s">
+    <row r="243" spans="1:2">
+      <c r="A243" t="s">
         <v>536</v>
       </c>
-      <c r="B239" t="str">
+      <c r="B243" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TRAILING : 'TRAILING' ;</v>
       </c>
     </row>
-    <row r="240" spans="1:2">
-      <c r="A240" t="s">
+    <row r="244" spans="1:2">
+      <c r="A244" t="s">
         <v>61</v>
       </c>
-      <c r="B240" t="str">
+      <c r="B244" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TRIGGER : 'TRIGGER' ;</v>
       </c>
     </row>
-    <row r="241" spans="1:2">
-      <c r="A241" s="2" t="s">
+    <row r="245" spans="1:2">
+      <c r="A245" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="B241" t="str">
+      <c r="B245" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>TRUE : 'TRUE' ;</v>
       </c>
     </row>
-    <row r="242" spans="1:2">
-      <c r="A242" t="s">
+    <row r="246" spans="1:2">
+      <c r="A246" t="s">
         <v>537</v>
       </c>
-      <c r="B242" t="str">
+      <c r="B246" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UNDO : 'UNDO' ;</v>
       </c>
     </row>
-    <row r="243" spans="1:2">
-      <c r="A243" t="s">
+    <row r="247" spans="1:2">
+      <c r="A247" t="s">
         <v>538</v>
       </c>
-      <c r="B243" t="str">
+      <c r="B247" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UNION : 'UNION' ;</v>
       </c>
     </row>
-    <row r="244" spans="1:2">
-      <c r="A244" t="s">
+    <row r="248" spans="1:2">
+      <c r="A248" t="s">
         <v>539</v>
       </c>
-      <c r="B244" t="str">
+      <c r="B248" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UNIQUE : 'UNIQUE' ;</v>
       </c>
     </row>
-    <row r="245" spans="1:2">
-      <c r="A245" t="s">
+    <row r="249" spans="1:2">
+      <c r="A249" t="s">
         <v>540</v>
       </c>
-      <c r="B245" t="str">
+      <c r="B249" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UNLOCK : 'UNLOCK' ;</v>
       </c>
     </row>
-    <row r="246" spans="1:2">
-      <c r="A246" t="s">
+    <row r="250" spans="1:2">
+      <c r="A250" t="s">
         <v>541</v>
       </c>
-      <c r="B246" t="str">
+      <c r="B250" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UNSIGNED : 'UNSIGNED' ;</v>
       </c>
     </row>
-    <row r="247" spans="1:2">
-      <c r="A247" t="s">
+    <row r="251" spans="1:2">
+      <c r="A251" t="s">
         <v>542</v>
       </c>
-      <c r="B247" t="str">
+      <c r="B251" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UPDATE : 'UPDATE' ;</v>
       </c>
     </row>
-    <row r="248" spans="1:2">
-      <c r="A248" t="s">
+    <row r="252" spans="1:2">
+      <c r="A252" t="s">
         <v>543</v>
       </c>
-      <c r="B248" t="str">
+      <c r="B252" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>USAGE : 'USAGE' ;</v>
       </c>
     </row>
-    <row r="249" spans="1:2">
-      <c r="A249" t="s">
+    <row r="253" spans="1:2">
+      <c r="A253" t="s">
         <v>544</v>
       </c>
-      <c r="B249" t="str">
+      <c r="B253" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>USE : 'USE' ;</v>
       </c>
     </row>
-    <row r="250" spans="1:2">
-      <c r="A250" t="s">
+    <row r="254" spans="1:2">
+      <c r="A254" t="s">
+        <v>63</v>
+      </c>
+      <c r="B254" s="3" t="str">
+        <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
+        <v>USER : 'USER' ;</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" t="s">
         <v>545</v>
       </c>
-      <c r="B250" t="str">
+      <c r="B255" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>USING : 'USING' ;</v>
       </c>
     </row>
-    <row r="251" spans="1:2">
-      <c r="A251" t="s">
+    <row r="256" spans="1:2">
+      <c r="A256" t="s">
         <v>546</v>
       </c>
-      <c r="B251" t="str">
+      <c r="B256" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UTC_DATE : 'UTC_DATE' ;</v>
       </c>
     </row>
-    <row r="252" spans="1:2">
-      <c r="A252" t="s">
+    <row r="257" spans="1:2">
+      <c r="A257" t="s">
         <v>547</v>
       </c>
-      <c r="B252" t="str">
+      <c r="B257" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UTC_TIME : 'UTC_TIME' ;</v>
       </c>
     </row>
-    <row r="253" spans="1:2">
-      <c r="A253" t="s">
+    <row r="258" spans="1:2">
+      <c r="A258" t="s">
         <v>548</v>
       </c>
-      <c r="B253" t="str">
+      <c r="B258" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>UTC_TIMESTAMP : 'UTC_TIMESTAMP' ;</v>
       </c>
     </row>
-    <row r="254" spans="1:2">
-      <c r="A254" t="s">
+    <row r="259" spans="1:2">
+      <c r="A259" t="s">
         <v>549</v>
       </c>
-      <c r="B254" t="str">
+      <c r="B259" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VALUES : 'VALUES' ;</v>
       </c>
     </row>
-    <row r="255" spans="1:2">
-      <c r="A255" t="s">
+    <row r="260" spans="1:2">
+      <c r="A260" t="s">
         <v>550</v>
       </c>
-      <c r="B255" t="str">
+      <c r="B260" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VARBINARY : 'VARBINARY' ;</v>
       </c>
     </row>
-    <row r="256" spans="1:2">
-      <c r="A256" t="s">
+    <row r="261" spans="1:2">
+      <c r="A261" t="s">
         <v>551</v>
       </c>
-      <c r="B256" t="str">
+      <c r="B261" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VARCHAR : 'VARCHAR' ;</v>
       </c>
     </row>
-    <row r="257" spans="1:2">
-      <c r="A257" t="s">
+    <row r="262" spans="1:2">
+      <c r="A262" t="s">
         <v>552</v>
       </c>
-      <c r="B257" t="str">
+      <c r="B262" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VARCHARACTER : 'VARCHARACTER' ;</v>
       </c>
     </row>
-    <row r="258" spans="1:2">
-      <c r="A258" t="s">
+    <row r="263" spans="1:2">
+      <c r="A263" t="s">
         <v>553</v>
       </c>
-      <c r="B258" t="str">
+      <c r="B263" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VARYING : 'VARYING' ;</v>
       </c>
     </row>
-    <row r="259" spans="1:2">
-      <c r="A259" t="s">
+    <row r="264" spans="1:2">
+      <c r="A264" t="s">
         <v>565</v>
       </c>
-      <c r="B259" t="str">
+      <c r="B264" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VECTOR : 'VECTOR' ;</v>
       </c>
     </row>
-    <row r="260" spans="1:2">
-      <c r="A260" t="s">
+    <row r="265" spans="1:2">
+      <c r="A265" t="s">
         <v>584</v>
       </c>
-      <c r="B260" s="3" t="str">
+      <c r="B265" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>VIA : 'VIA' ;</v>
       </c>
     </row>
-    <row r="261" spans="1:2">
-      <c r="A261" t="s">
+    <row r="266" spans="1:2">
+      <c r="A266" t="s">
         <v>554</v>
       </c>
-      <c r="B261" t="str">
+      <c r="B266" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WHEN : 'WHEN' ;</v>
       </c>
     </row>
-    <row r="262" spans="1:2">
-      <c r="A262" t="s">
+    <row r="267" spans="1:2">
+      <c r="A267" t="s">
         <v>555</v>
       </c>
-      <c r="B262" t="str">
+      <c r="B267" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WHERE : 'WHERE' ;</v>
       </c>
     </row>
-    <row r="263" spans="1:2">
-      <c r="A263" t="s">
+    <row r="268" spans="1:2">
+      <c r="A268" t="s">
         <v>556</v>
       </c>
-      <c r="B263" t="str">
+      <c r="B268" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WHILE : 'WHILE' ;</v>
       </c>
     </row>
-    <row r="264" spans="1:2">
-      <c r="A264" t="s">
+    <row r="269" spans="1:2">
+      <c r="A269" t="s">
         <v>557</v>
       </c>
-      <c r="B264" t="str">
+      <c r="B269" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WINDOW : 'WINDOW' ;</v>
       </c>
     </row>
-    <row r="265" spans="1:2">
-      <c r="A265" t="s">
+    <row r="270" spans="1:2">
+      <c r="A270" t="s">
         <v>558</v>
       </c>
-      <c r="B265" t="str">
+      <c r="B270" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WITH : 'WITH' ;</v>
       </c>
     </row>
-    <row r="266" spans="1:2">
-      <c r="A266" t="s">
+    <row r="271" spans="1:2">
+      <c r="A271" t="s">
         <v>559</v>
       </c>
-      <c r="B266" t="str">
+      <c r="B271" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>WRITE : 'WRITE' ;</v>
       </c>
     </row>
-    <row r="267" spans="1:2">
-      <c r="A267" t="s">
+    <row r="272" spans="1:2">
+      <c r="A272" t="s">
         <v>572</v>
       </c>
-      <c r="B267" s="3" t="str">
+      <c r="B272" s="3" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>X509 : 'X509' ;</v>
       </c>
     </row>
-    <row r="268" spans="1:2">
-      <c r="A268" t="s">
+    <row r="273" spans="1:2">
+      <c r="A273" t="s">
         <v>560</v>
       </c>
-      <c r="B268" t="str">
+      <c r="B273" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>XOR : 'XOR' ;</v>
       </c>
     </row>
-    <row r="269" spans="1:2">
-      <c r="A269" t="s">
+    <row r="274" spans="1:2">
+      <c r="A274" t="s">
         <v>561</v>
       </c>
-      <c r="B269" t="str">
+      <c r="B274" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>YEAR_MONTH : 'YEAR_MONTH' ;</v>
       </c>
     </row>
-    <row r="270" spans="1:2">
-      <c r="A270" t="s">
+    <row r="275" spans="1:2">
+      <c r="A275" t="s">
         <v>562</v>
       </c>
-      <c r="B270" t="str">
+      <c r="B275" t="str">
         <f>UPPER(Table3[[#This Row],[ACCOUNT]]) &amp; " : '"&amp; UPPER(Table3[[#This Row],[ACCOUNT]]) &amp;"' ;"</f>
         <v>ZEROFILL : 'ZEROFILL' ;</v>
       </c>

</xml_diff>